<commit_message>
Refresh dashboard with updated data
</commit_message>
<xml_diff>
--- a/outputs/templates_donnees_dashboard_MVE.xlsx
+++ b/outputs/templates_donnees_dashboard_MVE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Préparation EBOLA\SitReps\Data surveillance\analyse_poe\analyse_poe\CAR_Dashboard_Preparation_Menace_MVE\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE771361-5ACA-4783-AEF6-C94C16D3CBAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBCDECB-86F0-442E-8EEF-FDB93405E179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="contexte" sheetId="1" r:id="rId1"/>
@@ -832,7 +832,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2758,7 +2758,7 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="4">
-        <v>46196</v>
+        <v>46185</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>202</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="4">
-        <v>46196</v>
+        <v>46186</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>202</v>
@@ -2826,7 +2826,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="4">
-        <v>46196</v>
+        <v>46187</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>202</v>
@@ -2858,7 +2858,7 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="4">
-        <v>46196</v>
+        <v>46188</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>202</v>
@@ -2890,7 +2890,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="4">
-        <v>46196</v>
+        <v>46189</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>202</v>
@@ -2922,7 +2922,7 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="4">
-        <v>46196</v>
+        <v>46190</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>202</v>
@@ -2954,7 +2954,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="4">
-        <v>46196</v>
+        <v>46191</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>202</v>
@@ -2986,7 +2986,7 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="4">
-        <v>46196</v>
+        <v>46192</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>202</v>
@@ -3018,7 +3018,7 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="4">
-        <v>46196</v>
+        <v>46193</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>202</v>
@@ -3050,7 +3050,7 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="4">
-        <v>46196</v>
+        <v>46194</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>202</v>
@@ -3082,7 +3082,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="4">
-        <v>46196</v>
+        <v>46195</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>202</v>
@@ -3370,7 +3370,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4">
-        <v>46196</v>
+        <v>46185</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>202</v>
@@ -3402,7 +3402,7 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4">
-        <v>46196</v>
+        <v>46186</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>202</v>
@@ -3434,7 +3434,7 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4">
-        <v>46196</v>
+        <v>46187</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>202</v>
@@ -3466,7 +3466,7 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4">
-        <v>46196</v>
+        <v>46188</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>202</v>
@@ -3498,7 +3498,7 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4">
-        <v>46196</v>
+        <v>46189</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>202</v>
@@ -3530,7 +3530,7 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4">
-        <v>46196</v>
+        <v>46190</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>202</v>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4">
-        <v>46196</v>
+        <v>46191</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>202</v>
@@ -3594,7 +3594,7 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4">
-        <v>46196</v>
+        <v>46192</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>202</v>
@@ -3626,7 +3626,7 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4">
-        <v>46196</v>
+        <v>46184</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>202</v>
@@ -3658,7 +3658,7 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4">
-        <v>46196</v>
+        <v>46185</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>202</v>
@@ -3690,7 +3690,7 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4">
-        <v>46196</v>
+        <v>46186</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>202</v>
@@ -3722,7 +3722,7 @@
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4">
-        <v>46196</v>
+        <v>46187</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>202</v>
@@ -3754,7 +3754,7 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4">
-        <v>46196</v>
+        <v>46188</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>202</v>
@@ -3786,7 +3786,7 @@
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4">
-        <v>46196</v>
+        <v>46189</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>202</v>
@@ -3818,7 +3818,7 @@
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4">
-        <v>46196</v>
+        <v>46190</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>202</v>
@@ -3850,7 +3850,7 @@
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4">
-        <v>46196</v>
+        <v>46191</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>202</v>
@@ -3882,7 +3882,7 @@
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4">
-        <v>46196</v>
+        <v>46191</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>202</v>
@@ -3914,7 +3914,7 @@
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4">
-        <v>46196</v>
+        <v>46193</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>202</v>
@@ -3946,7 +3946,7 @@
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4">
-        <v>46196</v>
+        <v>46194</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>202</v>
@@ -4010,7 +4010,7 @@
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4">
-        <v>46196</v>
+        <v>46184</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>202</v>
@@ -4042,7 +4042,7 @@
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4">
-        <v>46196</v>
+        <v>46185</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>202</v>
@@ -4074,7 +4074,7 @@
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4">
-        <v>46196</v>
+        <v>46186</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>202</v>
@@ -4106,7 +4106,7 @@
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4">
-        <v>46196</v>
+        <v>46187</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>202</v>
@@ -4138,7 +4138,7 @@
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4">
-        <v>46196</v>
+        <v>46188</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>202</v>
@@ -4170,7 +4170,7 @@
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4">
-        <v>46196</v>
+        <v>46189</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>202</v>
@@ -4202,7 +4202,7 @@
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4">
-        <v>46196</v>
+        <v>46190</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>202</v>
@@ -4266,7 +4266,7 @@
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4">
-        <v>46196</v>
+        <v>46191</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>202</v>
@@ -4298,7 +4298,7 @@
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4">
-        <v>46196</v>
+        <v>46192</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>202</v>
@@ -4330,7 +4330,7 @@
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4">
-        <v>46196</v>
+        <v>46193</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>202</v>
@@ -4362,7 +4362,7 @@
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4">
-        <v>46196</v>
+        <v>46194</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>202</v>
@@ -4394,7 +4394,7 @@
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4">
-        <v>46196</v>
+        <v>46195</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>202</v>
@@ -4426,7 +4426,7 @@
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4">
-        <v>46196</v>
+        <v>46193</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>202</v>
@@ -4458,7 +4458,7 @@
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4">
-        <v>46196</v>
+        <v>46194</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>202</v>
@@ -4490,7 +4490,7 @@
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4">
-        <v>46196</v>
+        <v>46195</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>202</v>
@@ -4554,7 +4554,7 @@
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>202</v>
@@ -4586,7 +4586,7 @@
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>202</v>
@@ -6794,7 +6794,7 @@
     </row>
     <row r="128" spans="1:10">
       <c r="A128" s="4">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="B128" t="s">
         <v>202</v>
@@ -6825,7 +6825,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L128" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>